<commit_message>
ajout plan a 5 ans
</commit_message>
<xml_diff>
--- a/dataset_bi/finances_publiques_mel.xlsx
+++ b/dataset_bi/finances_publiques_mel.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U96"/>
+  <dimension ref="A1:X96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,6 +534,21 @@
           <t>solde_MEL</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>produit_FPB</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>tx_FPB</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>base_FPB</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -611,6 +626,15 @@
       <c r="U2" t="n">
         <v>232674</v>
       </c>
+      <c r="V2" t="n">
+        <v>69062</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="X2" t="n">
+        <v>106249.2307692308</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -688,6 +712,15 @@
       <c r="U3" t="n">
         <v>985251</v>
       </c>
+      <c r="V3" t="n">
+        <v>142190.47</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1.2247</v>
+      </c>
+      <c r="X3" t="n">
+        <v>116102.2862741896</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -765,6 +798,15 @@
       <c r="U4" t="n">
         <v>171778</v>
       </c>
+      <c r="V4" t="n">
+        <v>28787.99</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.5299</v>
+      </c>
+      <c r="X4" t="n">
+        <v>54327.21268163804</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -780,7 +822,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Armentières 59280,France</t>
+          <t>Armentières France</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -841,6 +883,15 @@
       </c>
       <c r="U5" t="n">
         <v>4955517</v>
+      </c>
+      <c r="V5" t="n">
+        <v>52828.65</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.5165</v>
+      </c>
+      <c r="X5" t="n">
+        <v>102281.9941916747</v>
       </c>
     </row>
     <row r="6">
@@ -919,6 +970,15 @@
       <c r="U6" t="n">
         <v>228050</v>
       </c>
+      <c r="V6" t="n">
+        <v>114280.12</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.4312</v>
+      </c>
+      <c r="X6" t="n">
+        <v>265028.107606679</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -996,6 +1056,15 @@
       <c r="U7" t="n">
         <v>449833</v>
       </c>
+      <c r="V7" t="n">
+        <v>129022.39</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0.4139</v>
+      </c>
+      <c r="X7" t="n">
+        <v>311723.5805750181</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1073,6 +1142,15 @@
       <c r="U8" t="n">
         <v>430534</v>
       </c>
+      <c r="V8" t="n">
+        <v>49028.25999999999</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.9626</v>
+      </c>
+      <c r="X8" t="n">
+        <v>50933.16019114896</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1150,6 +1228,15 @@
       <c r="U9" t="n">
         <v>101853</v>
       </c>
+      <c r="V9" t="n">
+        <v>68122.63</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.3963</v>
+      </c>
+      <c r="X9" t="n">
+        <v>171896.6187231895</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1227,6 +1314,15 @@
       <c r="U10" t="n">
         <v>280121</v>
       </c>
+      <c r="V10" t="n">
+        <v>107225.86</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.4386</v>
+      </c>
+      <c r="X10" t="n">
+        <v>244473.0050159599</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1304,6 +1400,15 @@
       <c r="U11" t="n">
         <v>1747822</v>
       </c>
+      <c r="V11" t="n">
+        <v>277543.45</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.4945000000000001</v>
+      </c>
+      <c r="X11" t="n">
+        <v>561260.7684529828</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1381,6 +1486,15 @@
       <c r="U12" t="n">
         <v>1178876</v>
       </c>
+      <c r="V12" t="n">
+        <v>88830.31</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.6031</v>
+      </c>
+      <c r="X12" t="n">
+        <v>147289.5208091527</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1458,6 +1572,15 @@
       <c r="U13" t="n">
         <v>83385</v>
       </c>
+      <c r="V13" t="n">
+        <v>33682.63</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.4163</v>
+      </c>
+      <c r="X13" t="n">
+        <v>80909.5123708864</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1535,6 +1658,15 @@
       <c r="U14" t="n">
         <v>216453</v>
       </c>
+      <c r="V14" t="n">
+        <v>22650.27</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.4327</v>
+      </c>
+      <c r="X14" t="n">
+        <v>52346.36006470996</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1612,6 +1744,15 @@
       <c r="U15" t="n">
         <v>83004</v>
       </c>
+      <c r="V15" t="n">
+        <v>33111.19</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.5619</v>
+      </c>
+      <c r="X15" t="n">
+        <v>58927.19345079197</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1689,6 +1830,15 @@
       <c r="U16" t="n">
         <v>414990</v>
       </c>
+      <c r="V16" t="n">
+        <v>48883.11</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.5911</v>
+      </c>
+      <c r="X16" t="n">
+        <v>82698.54508543394</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1766,6 +1916,15 @@
       <c r="U17" t="n">
         <v>2122016</v>
       </c>
+      <c r="V17" t="n">
+        <v>271856.76</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.6776000000000001</v>
+      </c>
+      <c r="X17" t="n">
+        <v>401205.3719008264</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1843,6 +2002,15 @@
       <c r="U18" t="n">
         <v>3738845</v>
       </c>
+      <c r="V18" t="n">
+        <v>130149.3</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="X18" t="n">
+        <v>459891.5194346289</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1920,6 +2088,15 @@
       <c r="U19" t="n">
         <v>235785</v>
       </c>
+      <c r="V19" t="n">
+        <v>125322.04</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.4604</v>
+      </c>
+      <c r="X19" t="n">
+        <v>272202.5195482189</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1997,6 +2174,15 @@
       <c r="U20" t="n">
         <v>134751</v>
       </c>
+      <c r="V20" t="n">
+        <v>17239.93</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.5293</v>
+      </c>
+      <c r="X20" t="n">
+        <v>32571.18836198753</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2004,7 +2190,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Emmerin Hauts-de-France,France</t>
+          <t>Emmerin, France</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2054,7 +2240,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Emmerin Hauts-de-France,France, France</t>
+          <t>Emmerin, France, France</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -2073,6 +2259,15 @@
       </c>
       <c r="U21" t="n">
         <v>406172</v>
+      </c>
+      <c r="V21" t="n">
+        <v>72884.01000000001</v>
+      </c>
+      <c r="W21" t="n">
+        <v>0.8801000000000001</v>
+      </c>
+      <c r="X21" t="n">
+        <v>82813.32803090558</v>
       </c>
     </row>
     <row r="22">
@@ -2151,6 +2346,15 @@
       <c r="U22" t="n">
         <v>304066</v>
       </c>
+      <c r="V22" t="n">
+        <v>10898.51</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0.3551</v>
+      </c>
+      <c r="X22" t="n">
+        <v>30691.38270909603</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2228,6 +2432,15 @@
       <c r="U23" t="n">
         <v>398298</v>
       </c>
+      <c r="V23" t="n">
+        <v>141980.62</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0.4061999999999999</v>
+      </c>
+      <c r="X23" t="n">
+        <v>349533.7764647957</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2305,6 +2518,15 @@
       <c r="U24" t="n">
         <v>944368</v>
       </c>
+      <c r="V24" t="n">
+        <v>112034.41</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.4641</v>
+      </c>
+      <c r="X24" t="n">
+        <v>241401.4436543849</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2382,6 +2604,15 @@
       <c r="U25" t="n">
         <v>72906</v>
       </c>
+      <c r="V25" t="n">
+        <v>22369.08</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.4108</v>
+      </c>
+      <c r="X25" t="n">
+        <v>54452.4829600779</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2459,6 +2690,15 @@
       <c r="U26" t="n">
         <v>49068</v>
       </c>
+      <c r="V26" t="n">
+        <v>26078.74</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.4974</v>
+      </c>
+      <c r="X26" t="n">
+        <v>52430.11660635304</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2536,6 +2776,15 @@
       <c r="U27" t="n">
         <v>3006002</v>
       </c>
+      <c r="V27" t="n">
+        <v>172292.6</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="X27" t="n">
+        <v>309878.7769784172</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2613,6 +2862,15 @@
       <c r="U28" t="n">
         <v>101831</v>
       </c>
+      <c r="V28" t="n">
+        <v>7551</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="X28" t="n">
+        <v>15731.25</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2690,6 +2948,15 @@
       <c r="U29" t="n">
         <v>274881</v>
       </c>
+      <c r="V29" t="n">
+        <v>109378.55</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.4055</v>
+      </c>
+      <c r="X29" t="n">
+        <v>269737.4845869297</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2767,6 +3034,15 @@
       <c r="U30" t="n">
         <v>169042</v>
       </c>
+      <c r="V30" t="n">
+        <v>151309.9</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="X30" t="n">
+        <v>379222.8070175439</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2844,6 +3120,15 @@
       <c r="U31" t="n">
         <v>1991063</v>
       </c>
+      <c r="V31" t="n">
+        <v>129417.77</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.3677</v>
+      </c>
+      <c r="X31" t="n">
+        <v>351965.6513462061</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2921,6 +3206,15 @@
       <c r="U32" t="n">
         <v>71435</v>
       </c>
+      <c r="V32" t="n">
+        <v>97013.89</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0.3389</v>
+      </c>
+      <c r="X32" t="n">
+        <v>286261.1094718206</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2998,6 +3292,15 @@
       <c r="U33" t="n">
         <v>323153</v>
       </c>
+      <c r="V33" t="n">
+        <v>51072.67</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0.6667000000000001</v>
+      </c>
+      <c r="X33" t="n">
+        <v>76605.17474126292</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3075,6 +3378,15 @@
       <c r="U34" t="n">
         <v>618836</v>
       </c>
+      <c r="V34" t="n">
+        <v>61413.43</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0.7943000000000001</v>
+      </c>
+      <c r="X34" t="n">
+        <v>77317.67594108019</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3152,6 +3464,15 @@
       <c r="U35" t="n">
         <v>2501164</v>
       </c>
+      <c r="V35" t="n">
+        <v>179899.4</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="X35" t="n">
+        <v>349998.8326848249</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3229,6 +3550,15 @@
       <c r="U36" t="n">
         <v>172662</v>
       </c>
+      <c r="V36" t="n">
+        <v>38350.25999999999</v>
+      </c>
+      <c r="W36" t="n">
+        <v>1.0626</v>
+      </c>
+      <c r="X36" t="n">
+        <v>36090.96555618294</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3306,6 +3636,15 @@
       <c r="U37" t="n">
         <v>2885473</v>
       </c>
+      <c r="V37" t="n">
+        <v>59673.44</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0.7444</v>
+      </c>
+      <c r="X37" t="n">
+        <v>80163.13809779689</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3383,6 +3722,15 @@
       <c r="U38" t="n">
         <v>2639319</v>
       </c>
+      <c r="V38" t="n">
+        <v>135515.9</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="X38" t="n">
+        <v>218927.140549273</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3460,6 +3808,15 @@
       <c r="U39" t="n">
         <v>494481</v>
       </c>
+      <c r="V39" t="n">
+        <v>99708.05</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0.4905</v>
+      </c>
+      <c r="X39" t="n">
+        <v>203278.3893985729</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3537,6 +3894,15 @@
       <c r="U40" t="n">
         <v>527151</v>
       </c>
+      <c r="V40" t="n">
+        <v>94984.14</v>
+      </c>
+      <c r="W40" t="n">
+        <v>0.7314000000000001</v>
+      </c>
+      <c r="X40" t="n">
+        <v>129866.201804758</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3614,6 +3980,15 @@
       <c r="U41" t="n">
         <v>340055</v>
       </c>
+      <c r="V41" t="n">
+        <v>150070.96</v>
+      </c>
+      <c r="W41" t="n">
+        <v>0.5396</v>
+      </c>
+      <c r="X41" t="n">
+        <v>278115.1964418088</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3691,6 +4066,15 @@
       <c r="U42" t="n">
         <v>213784</v>
       </c>
+      <c r="V42" t="n">
+        <v>130298.72</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0.6972</v>
+      </c>
+      <c r="X42" t="n">
+        <v>186888.5829030407</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3768,6 +4152,15 @@
       <c r="U43" t="n">
         <v>797829</v>
       </c>
+      <c r="V43" t="n">
+        <v>41918.9</v>
+      </c>
+      <c r="W43" t="n">
+        <v>0.5489999999999999</v>
+      </c>
+      <c r="X43" t="n">
+        <v>76355.00910746814</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3845,6 +4238,15 @@
       <c r="U44" t="n">
         <v>923724</v>
       </c>
+      <c r="V44" t="n">
+        <v>137887.69</v>
+      </c>
+      <c r="W44" t="n">
+        <v>0.5069</v>
+      </c>
+      <c r="X44" t="n">
+        <v>272021.4835273229</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3922,6 +4324,15 @@
       <c r="U45" t="n">
         <v>2511724</v>
       </c>
+      <c r="V45" t="n">
+        <v>79831.66</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0.1366</v>
+      </c>
+      <c r="X45" t="n">
+        <v>584419.1800878478</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3999,6 +4410,15 @@
       <c r="U46" t="n">
         <v>9798672</v>
       </c>
+      <c r="V46" t="n">
+        <v>100870.53</v>
+      </c>
+      <c r="W46" t="n">
+        <v>0.4353</v>
+      </c>
+      <c r="X46" t="n">
+        <v>231726.4645072364</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -4076,6 +4496,15 @@
       <c r="U47" t="n">
         <v>223723</v>
       </c>
+      <c r="V47" t="n">
+        <v>1776.79</v>
+      </c>
+      <c r="W47" t="n">
+        <v>0.5478999999999999</v>
+      </c>
+      <c r="X47" t="n">
+        <v>3242.909290016426</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -4153,6 +4582,15 @@
       <c r="U48" t="n">
         <v>78441</v>
       </c>
+      <c r="V48" t="n">
+        <v>46673.8</v>
+      </c>
+      <c r="W48" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="X48" t="n">
+        <v>90103.86100386101</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -4230,6 +4668,15 @@
       <c r="U49" t="n">
         <v>1112189</v>
       </c>
+      <c r="V49" t="n">
+        <v>73318.28</v>
+      </c>
+      <c r="W49" t="n">
+        <v>0.6228</v>
+      </c>
+      <c r="X49" t="n">
+        <v>117723.6351958895</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4307,6 +4754,15 @@
       <c r="U50" t="n">
         <v>2570626</v>
       </c>
+      <c r="V50" t="n">
+        <v>87855.20999999999</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0.4721</v>
+      </c>
+      <c r="X50" t="n">
+        <v>186094.4926922262</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4384,6 +4840,15 @@
       <c r="U51" t="n">
         <v>718722</v>
       </c>
+      <c r="V51" t="n">
+        <v>82185.89</v>
+      </c>
+      <c r="W51" t="n">
+        <v>0.5989</v>
+      </c>
+      <c r="X51" t="n">
+        <v>137228.0681248957</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -4461,6 +4926,15 @@
       <c r="U52" t="n">
         <v>47667164</v>
       </c>
+      <c r="V52" t="n">
+        <v>1296993.65</v>
+      </c>
+      <c r="W52" t="n">
+        <v>0.1665</v>
+      </c>
+      <c r="X52" t="n">
+        <v>7789751.651651652</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4538,6 +5012,15 @@
       <c r="U53" t="n">
         <v>1059482</v>
       </c>
+      <c r="V53" t="n">
+        <v>198723.78</v>
+      </c>
+      <c r="W53" t="n">
+        <v>0.6378</v>
+      </c>
+      <c r="X53" t="n">
+        <v>311576.9520225776</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4615,6 +5098,15 @@
       <c r="U54" t="n">
         <v>362806</v>
       </c>
+      <c r="V54" t="n">
+        <v>43806.39</v>
+      </c>
+      <c r="W54" t="n">
+        <v>0.5239</v>
+      </c>
+      <c r="X54" t="n">
+        <v>83615.93815613666</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4692,6 +5184,15 @@
       <c r="U55" t="n">
         <v>4725374</v>
       </c>
+      <c r="V55" t="n">
+        <v>81949.20999999999</v>
+      </c>
+      <c r="W55" t="n">
+        <v>0.7620999999999999</v>
+      </c>
+      <c r="X55" t="n">
+        <v>107530.7833617635</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4769,6 +5270,15 @@
       <c r="U56" t="n">
         <v>1890929</v>
       </c>
+      <c r="V56" t="n">
+        <v>34395.69</v>
+      </c>
+      <c r="W56" t="n">
+        <v>0.5468999999999999</v>
+      </c>
+      <c r="X56" t="n">
+        <v>62892.10093252881</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4846,6 +5356,15 @@
       <c r="U57" t="n">
         <v>7567103</v>
       </c>
+      <c r="V57" t="n">
+        <v>236414.19</v>
+      </c>
+      <c r="W57" t="n">
+        <v>0.1919</v>
+      </c>
+      <c r="X57" t="n">
+        <v>1231965.55497655</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4923,6 +5442,15 @@
       <c r="U58" t="n">
         <v>2082314</v>
       </c>
+      <c r="V58" t="n">
+        <v>190193.32</v>
+      </c>
+      <c r="W58" t="n">
+        <v>0.6431999999999999</v>
+      </c>
+      <c r="X58" t="n">
+        <v>295698.5696517414</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -5000,6 +5528,15 @@
       <c r="U59" t="n">
         <v>282116</v>
       </c>
+      <c r="V59" t="n">
+        <v>100553.32</v>
+      </c>
+      <c r="W59" t="n">
+        <v>0.5632</v>
+      </c>
+      <c r="X59" t="n">
+        <v>178539.2755681818</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -5077,6 +5614,15 @@
       <c r="U60" t="n">
         <v>1034932</v>
       </c>
+      <c r="V60" t="n">
+        <v>32415.85</v>
+      </c>
+      <c r="W60" t="n">
+        <v>0.4885</v>
+      </c>
+      <c r="X60" t="n">
+        <v>66357.93244626407</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -5154,6 +5700,15 @@
       <c r="U61" t="n">
         <v>3492614</v>
       </c>
+      <c r="V61" t="n">
+        <v>121918.12</v>
+      </c>
+      <c r="W61" t="n">
+        <v>0.8912</v>
+      </c>
+      <c r="X61" t="n">
+        <v>136802.1992818671</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -5231,6 +5786,15 @@
       <c r="U62" t="n">
         <v>854320</v>
       </c>
+      <c r="V62" t="n">
+        <v>53613.38</v>
+      </c>
+      <c r="W62" t="n">
+        <v>0.4838</v>
+      </c>
+      <c r="X62" t="n">
+        <v>110817.2385283175</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -5308,6 +5872,15 @@
       <c r="U63" t="n">
         <v>1211053</v>
       </c>
+      <c r="V63" t="n">
+        <v>19946.06</v>
+      </c>
+      <c r="W63" t="n">
+        <v>0.3806</v>
+      </c>
+      <c r="X63" t="n">
+        <v>52406.8838675775</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -5385,6 +5958,15 @@
       <c r="U64" t="n">
         <v>1070341</v>
       </c>
+      <c r="V64" t="n">
+        <v>30117.88</v>
+      </c>
+      <c r="W64" t="n">
+        <v>0.7787999999999999</v>
+      </c>
+      <c r="X64" t="n">
+        <v>38672.16230097586</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -5462,6 +6044,15 @@
       <c r="U65" t="n">
         <v>179889</v>
       </c>
+      <c r="V65" t="n">
+        <v>10941.65</v>
+      </c>
+      <c r="W65" t="n">
+        <v>0.6665000000000001</v>
+      </c>
+      <c r="X65" t="n">
+        <v>16416.57914478619</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -5539,6 +6130,15 @@
       <c r="U66" t="n">
         <v>156064</v>
       </c>
+      <c r="V66" t="n">
+        <v>79790.81</v>
+      </c>
+      <c r="W66" t="n">
+        <v>0.5981000000000001</v>
+      </c>
+      <c r="X66" t="n">
+        <v>133407.1392743688</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -5616,6 +6216,15 @@
       <c r="U67" t="n">
         <v>455651</v>
       </c>
+      <c r="V67" t="n">
+        <v>36514.46</v>
+      </c>
+      <c r="W67" t="n">
+        <v>0.5546</v>
+      </c>
+      <c r="X67" t="n">
+        <v>65839.27154706094</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -5693,6 +6302,15 @@
       <c r="U68" t="n">
         <v>962684</v>
       </c>
+      <c r="V68" t="n">
+        <v>207351.71</v>
+      </c>
+      <c r="W68" t="n">
+        <v>0.6570999999999999</v>
+      </c>
+      <c r="X68" t="n">
+        <v>315555.7905950389</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -5770,6 +6388,15 @@
       <c r="U69" t="n">
         <v>89985</v>
       </c>
+      <c r="V69" t="n">
+        <v>76888.14</v>
+      </c>
+      <c r="W69" t="n">
+        <v>0.3114</v>
+      </c>
+      <c r="X69" t="n">
+        <v>246911.1753371869</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -5847,6 +6474,15 @@
       <c r="U70" t="n">
         <v>2507634</v>
       </c>
+      <c r="V70" t="n">
+        <v>133968.84</v>
+      </c>
+      <c r="W70" t="n">
+        <v>0.5884</v>
+      </c>
+      <c r="X70" t="n">
+        <v>227683.2766825289</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -5924,6 +6560,15 @@
       <c r="U71" t="n">
         <v>1239260</v>
       </c>
+      <c r="V71" t="n">
+        <v>143999.39</v>
+      </c>
+      <c r="W71" t="n">
+        <v>0.5239</v>
+      </c>
+      <c r="X71" t="n">
+        <v>274860.4504676465</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -6001,6 +6646,15 @@
       <c r="U72" t="n">
         <v>6015537</v>
       </c>
+      <c r="V72" t="n">
+        <v>300604.74</v>
+      </c>
+      <c r="W72" t="n">
+        <v>0.6074000000000001</v>
+      </c>
+      <c r="X72" t="n">
+        <v>494904.0829766216</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -6078,6 +6732,15 @@
       <c r="U73" t="n">
         <v>482126</v>
       </c>
+      <c r="V73" t="n">
+        <v>62794.06</v>
+      </c>
+      <c r="W73" t="n">
+        <v>0.5506</v>
+      </c>
+      <c r="X73" t="n">
+        <v>114046.603705049</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -6155,6 +6818,15 @@
       <c r="U74" t="n">
         <v>1702753</v>
       </c>
+      <c r="V74" t="n">
+        <v>132195.64</v>
+      </c>
+      <c r="W74" t="n">
+        <v>0.3664</v>
+      </c>
+      <c r="X74" t="n">
+        <v>360795.96069869</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -6232,6 +6904,15 @@
       <c r="U75" t="n">
         <v>626213</v>
       </c>
+      <c r="V75" t="n">
+        <v>115350.61</v>
+      </c>
+      <c r="W75" t="n">
+        <v>0.7361</v>
+      </c>
+      <c r="X75" t="n">
+        <v>156705.0808314088</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -6309,6 +6990,15 @@
       <c r="U76" t="n">
         <v>402232</v>
       </c>
+      <c r="V76" t="n">
+        <v>80396.39</v>
+      </c>
+      <c r="W76" t="n">
+        <v>0.9939</v>
+      </c>
+      <c r="X76" t="n">
+        <v>80889.81788912366</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -6386,6 +7076,15 @@
       <c r="U77" t="n">
         <v>333002</v>
       </c>
+      <c r="V77" t="n">
+        <v>68601.73999999999</v>
+      </c>
+      <c r="W77" t="n">
+        <v>0.5874</v>
+      </c>
+      <c r="X77" t="n">
+        <v>116788.7980932925</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -6463,6 +7162,15 @@
       <c r="U78" t="n">
         <v>1711342</v>
       </c>
+      <c r="V78" t="n">
+        <v>250266</v>
+      </c>
+      <c r="W78" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="X78" t="n">
+        <v>582013.9534883721</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -6540,6 +7248,15 @@
       <c r="U79" t="n">
         <v>1184968</v>
       </c>
+      <c r="V79" t="n">
+        <v>56813.13</v>
+      </c>
+      <c r="W79" t="n">
+        <v>0.6912999999999999</v>
+      </c>
+      <c r="X79" t="n">
+        <v>82183.03196875453</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -6617,6 +7334,15 @@
       <c r="U80" t="n">
         <v>3491557</v>
       </c>
+      <c r="V80" t="n">
+        <v>88688.2</v>
+      </c>
+      <c r="W80" t="n">
+        <v>0.302</v>
+      </c>
+      <c r="X80" t="n">
+        <v>293669.5364238411</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -6694,6 +7420,15 @@
       <c r="U81" t="n">
         <v>67188</v>
       </c>
+      <c r="V81" t="n">
+        <v>68306.31</v>
+      </c>
+      <c r="W81" t="n">
+        <v>0.4631</v>
+      </c>
+      <c r="X81" t="n">
+        <v>147497.9702008205</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -6771,6 +7506,15 @@
       <c r="U82" t="n">
         <v>784654</v>
       </c>
+      <c r="V82" t="n">
+        <v>19851.06</v>
+      </c>
+      <c r="W82" t="n">
+        <v>0.1706</v>
+      </c>
+      <c r="X82" t="n">
+        <v>116360.2579132474</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -6848,6 +7592,15 @@
       <c r="U83" t="n">
         <v>13827009</v>
       </c>
+      <c r="V83" t="n">
+        <v>213313.5</v>
+      </c>
+      <c r="W83" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="X83" t="n">
+        <v>430936.3636363636</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -6863,7 +7616,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Vendeville 59175,France</t>
+          <t>Vendeville France</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -6924,6 +7677,15 @@
       </c>
       <c r="U84" t="n">
         <v>100816</v>
+      </c>
+      <c r="V84" t="n">
+        <v>19006.04</v>
+      </c>
+      <c r="W84" t="n">
+        <v>0.6604000000000001</v>
+      </c>
+      <c r="X84" t="n">
+        <v>28779.58812840702</v>
       </c>
     </row>
     <row r="85">
@@ -7002,6 +7764,15 @@
       <c r="U85" t="n">
         <v>144221</v>
       </c>
+      <c r="V85" t="n">
+        <v>38416.18</v>
+      </c>
+      <c r="W85" t="n">
+        <v>0.6718000000000001</v>
+      </c>
+      <c r="X85" t="n">
+        <v>57183.95355760642</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -7079,6 +7850,15 @@
       <c r="U86" t="n">
         <v>299048</v>
       </c>
+      <c r="V86" t="n">
+        <v>131864.39</v>
+      </c>
+      <c r="W86" t="n">
+        <v>0.3639</v>
+      </c>
+      <c r="X86" t="n">
+        <v>362364.3583402034</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -7156,6 +7936,15 @@
       <c r="U87" t="n">
         <v>2478207</v>
       </c>
+      <c r="V87" t="n">
+        <v>476906.04</v>
+      </c>
+      <c r="W87" t="n">
+        <v>0.8704000000000001</v>
+      </c>
+      <c r="X87" t="n">
+        <v>547915.9466911765</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -7233,6 +8022,15 @@
       <c r="U88" t="n">
         <v>1799432</v>
       </c>
+      <c r="V88" t="n">
+        <v>245559</v>
+      </c>
+      <c r="W88" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="X88" t="n">
+        <v>438498.2142857143</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -7310,6 +8108,15 @@
       <c r="U89" t="n">
         <v>114501</v>
       </c>
+      <c r="V89" t="n">
+        <v>44952.62</v>
+      </c>
+      <c r="W89" t="n">
+        <v>0.2262</v>
+      </c>
+      <c r="X89" t="n">
+        <v>198729.5313881521</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -7387,6 +8194,15 @@
       <c r="U90" t="n">
         <v>3384176</v>
       </c>
+      <c r="V90" t="n">
+        <v>198148.56</v>
+      </c>
+      <c r="W90" t="n">
+        <v>0.5756</v>
+      </c>
+      <c r="X90" t="n">
+        <v>344246.9770674079</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -7464,6 +8280,15 @@
       <c r="U91" t="n">
         <v>2585708</v>
       </c>
+      <c r="V91" t="n">
+        <v>77651.48999999999</v>
+      </c>
+      <c r="W91" t="n">
+        <v>0.5449000000000001</v>
+      </c>
+      <c r="X91" t="n">
+        <v>142505.9460451459</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -7541,6 +8366,15 @@
       <c r="U92" t="n">
         <v>6149788</v>
       </c>
+      <c r="V92" t="n">
+        <v>338605.04</v>
+      </c>
+      <c r="W92" t="n">
+        <v>1.1304</v>
+      </c>
+      <c r="X92" t="n">
+        <v>299544.4444444444</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -7618,6 +8452,15 @@
       <c r="U93" t="n">
         <v>793327</v>
       </c>
+      <c r="V93" t="n">
+        <v>160861.61</v>
+      </c>
+      <c r="W93" t="n">
+        <v>0.5161</v>
+      </c>
+      <c r="X93" t="n">
+        <v>311686.9017632242</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -7695,6 +8538,15 @@
       <c r="U94" t="n">
         <v>953326</v>
       </c>
+      <c r="V94" t="n">
+        <v>92075.7</v>
+      </c>
+      <c r="W94" t="n">
+        <v>0.5770000000000001</v>
+      </c>
+      <c r="X94" t="n">
+        <v>159576.603119584</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -7772,6 +8624,15 @@
       <c r="U95" t="n">
         <v>97759</v>
       </c>
+      <c r="V95" t="n">
+        <v>44870.79</v>
+      </c>
+      <c r="W95" t="n">
+        <v>0.7179000000000001</v>
+      </c>
+      <c r="X95" t="n">
+        <v>62502.84162139573</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -7848,6 +8709,15 @@
       </c>
       <c r="U96" t="n">
         <v>442286</v>
+      </c>
+      <c r="V96" t="n">
+        <v>94616.01999999999</v>
+      </c>
+      <c r="W96" t="n">
+        <v>0.7302</v>
+      </c>
+      <c r="X96" t="n">
+        <v>129575.4861681731</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mise a jour des données a 5ans
</commit_message>
<xml_diff>
--- a/dataset_bi/finances_publiques_mel.xlsx
+++ b/dataset_bi/finances_publiques_mel.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LeWagon\Projet_crise_logement\dataset_bi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Formation\crise_immo\Projet_crise_logement\dataset_bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F957865-DEB8-46C8-9DBF-689F746A173E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="finances_2024" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="499">
   <si>
     <t>INSEE_x</t>
   </si>
@@ -1519,8 +1522,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1543,12 +1546,27 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -1565,6 +1583,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1573,10 +1599,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -1850,14 +1876,41 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:X96"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="29" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1931,7 +1984,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>59001</v>
       </c>
@@ -1954,7 +2007,7 @@
         <v>5</v>
       </c>
       <c r="H2">
-        <v>3157345.9700000002</v>
+        <v>3157345.97</v>
       </c>
       <c r="I2">
         <v>3421163.98</v>
@@ -1963,7 +2016,7 @@
         <v>263818.01000000018</v>
       </c>
       <c r="K2">
-        <v>3681561.2000000002</v>
+        <v>3681561.2</v>
       </c>
       <c r="L2">
         <v>7352</v>
@@ -1999,13 +2052,13 @@
         <v>69062</v>
       </c>
       <c r="W2">
-        <v>0.65000000000000002</v>
+        <v>0.65</v>
       </c>
       <c r="X2">
         <v>106249.23076923079</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>59008</v>
       </c>
@@ -2079,7 +2132,7 @@
         <v>116102.2862741896</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>59010</v>
       </c>
@@ -2111,7 +2164,7 @@
         <v>112990.4099999999</v>
       </c>
       <c r="K4">
-        <v>1796313.1899999999</v>
+        <v>1796313.19</v>
       </c>
       <c r="L4">
         <v>1707</v>
@@ -2144,7 +2197,7 @@
         <v>171778</v>
       </c>
       <c r="V4">
-        <v>28787.990000000002</v>
+        <v>28787.99</v>
       </c>
       <c r="W4">
         <v>0.52990000000000004</v>
@@ -2153,7 +2206,7 @@
         <v>54327.212681638041</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>59014</v>
       </c>
@@ -2218,7 +2271,7 @@
         <v>4955517</v>
       </c>
       <c r="V5">
-        <v>52828.650000000001</v>
+        <v>52828.65</v>
       </c>
       <c r="W5">
         <v>0.51649999999999996</v>
@@ -2227,7 +2280,7 @@
         <v>102281.9941916747</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>59017</v>
       </c>
@@ -2256,10 +2309,10 @@
         <v>1514403.97</v>
       </c>
       <c r="J6">
-        <v>449752.21999999997</v>
+        <v>449752.22</v>
       </c>
       <c r="K6">
-        <v>2371065.3100000001</v>
+        <v>2371065.31</v>
       </c>
       <c r="L6">
         <v>29201</v>
@@ -2301,7 +2354,7 @@
         <v>265028.10760667903</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>59043</v>
       </c>
@@ -2324,10 +2377,10 @@
         <v>44</v>
       </c>
       <c r="H7">
-        <v>4392581.5700000003</v>
+        <v>4392581.57</v>
       </c>
       <c r="I7">
-        <v>4910279.3399999999</v>
+        <v>4910279.34</v>
       </c>
       <c r="J7">
         <v>517697.76999999961</v>
@@ -2375,7 +2428,7 @@
         <v>311723.58057501807</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>59046</v>
       </c>
@@ -2398,7 +2451,7 @@
         <v>52</v>
       </c>
       <c r="H8">
-        <v>4327916.0700000003</v>
+        <v>4327916.07</v>
       </c>
       <c r="I8">
         <v>4860750.21</v>
@@ -2407,7 +2460,7 @@
         <v>532834.13999999966</v>
       </c>
       <c r="K8">
-        <v>5038293.0800000001</v>
+        <v>5038293.08</v>
       </c>
       <c r="L8">
         <v>79415</v>
@@ -2449,7 +2502,7 @@
         <v>50933.160191148963</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>59056</v>
       </c>
@@ -2472,7 +2525,7 @@
         <v>56</v>
       </c>
       <c r="H9">
-        <v>550538.40000000002</v>
+        <v>550538.4</v>
       </c>
       <c r="I9">
         <v>703158.84000000008</v>
@@ -2481,7 +2534,7 @@
         <v>152620.44000000009</v>
       </c>
       <c r="K9">
-        <v>1354030.1599999999</v>
+        <v>1354030.16</v>
       </c>
       <c r="L9">
         <v>2976</v>
@@ -2514,7 +2567,7 @@
         <v>101853</v>
       </c>
       <c r="V9">
-        <v>68122.630000000005</v>
+        <v>68122.63</v>
       </c>
       <c r="W9">
         <v>0.39629999999999999</v>
@@ -2523,7 +2576,7 @@
         <v>171896.61872318949</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>59067</v>
       </c>
@@ -2552,7 +2605,7 @@
         <v>1569908.46</v>
       </c>
       <c r="J10">
-        <v>102216.00999999999</v>
+        <v>102216.01</v>
       </c>
       <c r="K10">
         <v>3744816.79</v>
@@ -2597,7 +2650,7 @@
         <v>244473.0050159599</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>59088</v>
       </c>
@@ -2662,7 +2715,7 @@
         <v>1747822</v>
       </c>
       <c r="V11">
-        <v>277543.45000000001</v>
+        <v>277543.45</v>
       </c>
       <c r="W11">
         <v>0.49450000000000011</v>
@@ -2671,7 +2724,7 @@
         <v>561260.76845298277</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>59090</v>
       </c>
@@ -2700,7 +2753,7 @@
         <v>6275321.0800000001</v>
       </c>
       <c r="J12">
-        <v>594039.70999999996</v>
+        <v>594039.71</v>
       </c>
       <c r="K12">
         <v>8942130.8100000005</v>
@@ -2736,7 +2789,7 @@
         <v>1178876</v>
       </c>
       <c r="V12">
-        <v>88830.309999999998</v>
+        <v>88830.31</v>
       </c>
       <c r="W12">
         <v>0.60309999999999997</v>
@@ -2745,7 +2798,7 @@
         <v>147289.52080915269</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>59092</v>
       </c>
@@ -2768,7 +2821,7 @@
         <v>106</v>
       </c>
       <c r="H13">
-        <v>586127.85999999999</v>
+        <v>586127.86</v>
       </c>
       <c r="I13">
         <v>634428.88</v>
@@ -2819,7 +2872,7 @@
         <v>80909.512370886398</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>59128</v>
       </c>
@@ -2893,7 +2946,7 @@
         <v>52346.360064709959</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>59128</v>
       </c>
@@ -2919,13 +2972,13 @@
         <v>824755.94000000006</v>
       </c>
       <c r="I15">
-        <v>918846.03000000003</v>
+        <v>918846.03</v>
       </c>
       <c r="J15">
         <v>94090.089999999967</v>
       </c>
       <c r="K15">
-        <v>1358361.3200000001</v>
+        <v>1358361.32</v>
       </c>
       <c r="L15">
         <v>3785</v>
@@ -2958,7 +3011,7 @@
         <v>83004</v>
       </c>
       <c r="V15">
-        <v>33111.190000000002</v>
+        <v>33111.19</v>
       </c>
       <c r="W15">
         <v>0.56189999999999996</v>
@@ -2967,7 +3020,7 @@
         <v>58927.193450791972</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>59143</v>
       </c>
@@ -2990,10 +3043,10 @@
         <v>146</v>
       </c>
       <c r="H16">
-        <v>2641061.1600000001</v>
+        <v>2641061.16</v>
       </c>
       <c r="I16">
-        <v>2680953.5800000001</v>
+        <v>2680953.58</v>
       </c>
       <c r="J16">
         <v>39892.420000000391</v>
@@ -3032,7 +3085,7 @@
         <v>414990</v>
       </c>
       <c r="V16">
-        <v>48883.110000000001</v>
+        <v>48883.11</v>
       </c>
       <c r="W16">
         <v>0.59109999999999996</v>
@@ -3041,7 +3094,7 @@
         <v>82698.545085433943</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>59152</v>
       </c>
@@ -3070,7 +3123,7 @@
         <v>15407908.16</v>
       </c>
       <c r="J17">
-        <v>1229671.3200000001</v>
+        <v>1229671.32</v>
       </c>
       <c r="K17">
         <v>16423692.699999999</v>
@@ -3106,7 +3159,7 @@
         <v>2122016</v>
       </c>
       <c r="V17">
-        <v>271856.76000000001</v>
+        <v>271856.76</v>
       </c>
       <c r="W17">
         <v>0.67760000000000009</v>
@@ -3115,7 +3168,7 @@
         <v>401205.3719008264</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>59163</v>
       </c>
@@ -3189,7 +3242,7 @@
         <v>459891.51943462889</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>59173</v>
       </c>
@@ -3215,7 +3268,7 @@
         <v>1387418.98</v>
       </c>
       <c r="I19">
-        <v>1529617.5600000001</v>
+        <v>1529617.56</v>
       </c>
       <c r="J19">
         <v>142198.5800000001</v>
@@ -3254,7 +3307,7 @@
         <v>235785</v>
       </c>
       <c r="V19">
-        <v>125322.03999999999</v>
+        <v>125322.04</v>
       </c>
       <c r="W19">
         <v>0.46039999999999998</v>
@@ -3263,7 +3316,7 @@
         <v>272202.51954821887</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>59176</v>
       </c>
@@ -3286,7 +3339,7 @@
         <v>670</v>
       </c>
       <c r="H20">
-        <v>1343062.6899999999</v>
+        <v>1343062.69</v>
       </c>
       <c r="I20">
         <v>1307925.3600000001</v>
@@ -3295,7 +3348,7 @@
         <v>-35137.330000000067</v>
       </c>
       <c r="K20">
-        <v>1716036.5700000001</v>
+        <v>1716036.57</v>
       </c>
       <c r="L20">
         <v>903</v>
@@ -3337,7 +3390,7 @@
         <v>32571.18836198753</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>59193</v>
       </c>
@@ -3360,16 +3413,16 @@
         <v>193</v>
       </c>
       <c r="H21">
-        <v>2791447.7999999998</v>
+        <v>2791447.8</v>
       </c>
       <c r="I21">
-        <v>3141770.5800000001</v>
+        <v>3141770.58</v>
       </c>
       <c r="J21">
         <v>350322.78000000032</v>
       </c>
       <c r="K21">
-        <v>3635797.5699999998</v>
+        <v>3635797.57</v>
       </c>
       <c r="L21">
         <v>49584</v>
@@ -3411,7 +3464,7 @@
         <v>82813.328030905584</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>59194</v>
       </c>
@@ -3434,7 +3487,7 @@
         <v>195</v>
       </c>
       <c r="H22">
-        <v>808894.39000000001</v>
+        <v>808894.39</v>
       </c>
       <c r="I22">
         <v>1001849.77</v>
@@ -3443,7 +3496,7 @@
         <v>192955.38</v>
       </c>
       <c r="K22">
-        <v>3298806.9100000001</v>
+        <v>3298806.91</v>
       </c>
       <c r="L22">
         <v>2329</v>
@@ -3485,7 +3538,7 @@
         <v>30691.382709096029</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>59201</v>
       </c>
@@ -3508,16 +3561,16 @@
         <v>196</v>
       </c>
       <c r="H23">
-        <v>938275.14000000001</v>
+        <v>938275.14</v>
       </c>
       <c r="I23">
         <v>1241543.78</v>
       </c>
       <c r="J23">
-        <v>303268.64000000001</v>
+        <v>303268.64</v>
       </c>
       <c r="K23">
-        <v>4827789.4500000002</v>
+        <v>4827789.45</v>
       </c>
       <c r="L23">
         <v>6306</v>
@@ -3559,7 +3612,7 @@
         <v>349533.77646479569</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>59202</v>
       </c>
@@ -3582,7 +3635,7 @@
         <v>202</v>
       </c>
       <c r="H24">
-        <v>4841820.2999999998</v>
+        <v>4841820.3</v>
       </c>
       <c r="I24">
         <v>5506917.9500000002</v>
@@ -3633,7 +3686,7 @@
         <v>241401.4436543849</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>59203</v>
       </c>
@@ -3659,7 +3712,7 @@
         <v>400638</v>
       </c>
       <c r="I25">
-        <v>473035.09999999998</v>
+        <v>473035.1</v>
       </c>
       <c r="J25">
         <v>72397.099999999977</v>
@@ -3698,7 +3751,7 @@
         <v>72906</v>
       </c>
       <c r="V25">
-        <v>22369.080000000002</v>
+        <v>22369.08</v>
       </c>
       <c r="W25">
         <v>0.4108</v>
@@ -3707,7 +3760,7 @@
         <v>54452.482960077898</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>59206</v>
       </c>
@@ -3730,7 +3783,7 @@
         <v>208</v>
       </c>
       <c r="H26">
-        <v>244444.32000000001</v>
+        <v>244444.32</v>
       </c>
       <c r="I26">
         <v>250536.97</v>
@@ -3739,7 +3792,7 @@
         <v>6092.6499999999942</v>
       </c>
       <c r="K26">
-        <v>435615.53000000003</v>
+        <v>435615.53</v>
       </c>
       <c r="L26">
         <v>133</v>
@@ -3772,7 +3825,7 @@
         <v>49068</v>
       </c>
       <c r="V26">
-        <v>26078.740000000002</v>
+        <v>26078.74</v>
       </c>
       <c r="W26">
         <v>0.49740000000000001</v>
@@ -3781,7 +3834,7 @@
         <v>52430.11660635304</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>59220</v>
       </c>
@@ -3846,7 +3899,7 @@
         <v>3006002</v>
       </c>
       <c r="V27">
-        <v>172292.60000000001</v>
+        <v>172292.6</v>
       </c>
       <c r="W27">
         <v>0.55600000000000005</v>
@@ -3855,7 +3908,7 @@
         <v>309878.77697841718</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>59232</v>
       </c>
@@ -3878,7 +3931,7 @@
         <v>247</v>
       </c>
       <c r="H28">
-        <v>1360987.8999999999</v>
+        <v>1360987.9</v>
       </c>
       <c r="I28">
         <v>1365488.8</v>
@@ -3923,13 +3976,13 @@
         <v>7551</v>
       </c>
       <c r="W28">
-        <v>0.47999999999999998</v>
+        <v>0.48</v>
       </c>
       <c r="X28">
         <v>15731.25</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>59249</v>
       </c>
@@ -4003,7 +4056,7 @@
         <v>269737.48458692973</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>59255</v>
       </c>
@@ -4026,16 +4079,16 @@
         <v>252</v>
       </c>
       <c r="H30">
-        <v>2066053.3500000001</v>
+        <v>2066053.35</v>
       </c>
       <c r="I30">
-        <v>2312746.9399999999</v>
+        <v>2312746.94</v>
       </c>
       <c r="J30">
         <v>246693.58999999991</v>
       </c>
       <c r="K30">
-        <v>3469346.6000000001</v>
+        <v>3469346.6</v>
       </c>
       <c r="L30">
         <v>7419</v>
@@ -4068,7 +4121,7 @@
         <v>169042</v>
       </c>
       <c r="V30">
-        <v>151309.89999999999</v>
+        <v>151309.9</v>
       </c>
       <c r="W30">
         <v>0.39900000000000002</v>
@@ -4077,7 +4130,7 @@
         <v>379222.80701754388</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>59260</v>
       </c>
@@ -4100,7 +4153,7 @@
         <v>256</v>
       </c>
       <c r="H31">
-        <v>5161151.8200000003</v>
+        <v>5161151.82</v>
       </c>
       <c r="I31">
         <v>5518122.4500000002</v>
@@ -4151,7 +4204,7 @@
         <v>351965.65134620608</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>59261</v>
       </c>
@@ -4174,7 +4227,7 @@
         <v>257</v>
       </c>
       <c r="H32">
-        <v>767335.51000000001</v>
+        <v>767335.51</v>
       </c>
       <c r="I32">
         <v>796760.17999999993</v>
@@ -4183,7 +4236,7 @@
         <v>29424.669999999929</v>
       </c>
       <c r="K32">
-        <v>1416105.8899999999</v>
+        <v>1416105.89</v>
       </c>
       <c r="L32">
         <v>29934</v>
@@ -4216,7 +4269,7 @@
         <v>71435</v>
       </c>
       <c r="V32">
-        <v>97013.889999999999</v>
+        <v>97013.89</v>
       </c>
       <c r="W32">
         <v>0.33889999999999998</v>
@@ -4225,7 +4278,7 @@
         <v>286261.10947182059</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>59275</v>
       </c>
@@ -4251,7 +4304,7 @@
         <v>1125013.72</v>
       </c>
       <c r="I33">
-        <v>1368788.5700000001</v>
+        <v>1368788.57</v>
       </c>
       <c r="J33">
         <v>243774.84999999989</v>
@@ -4290,7 +4343,7 @@
         <v>323153</v>
       </c>
       <c r="V33">
-        <v>51072.669999999998</v>
+        <v>51072.67</v>
       </c>
       <c r="W33">
         <v>0.66670000000000007</v>
@@ -4299,7 +4352,7 @@
         <v>76605.174741262919</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>59286</v>
       </c>
@@ -4373,7 +4426,7 @@
         <v>77317.67594108019</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>59292</v>
       </c>
@@ -4402,7 +4455,7 @@
         <v>25060287.829999998</v>
       </c>
       <c r="J35">
-        <v>2585830.5899999999</v>
+        <v>2585830.59</v>
       </c>
       <c r="K35">
         <v>28760867.039999999</v>
@@ -4438,7 +4491,7 @@
         <v>2501164</v>
       </c>
       <c r="V35">
-        <v>179899.39999999999</v>
+        <v>179899.4</v>
       </c>
       <c r="W35">
         <v>0.51400000000000001</v>
@@ -4447,7 +4500,7 @@
         <v>349998.83268482488</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>59294</v>
       </c>
@@ -4470,7 +4523,7 @@
         <v>281</v>
       </c>
       <c r="H36">
-        <v>1011426.3199999999</v>
+        <v>1011426.32</v>
       </c>
       <c r="I36">
         <v>1096601.52</v>
@@ -4479,7 +4532,7 @@
         <v>85175.20000000007</v>
       </c>
       <c r="K36">
-        <v>1350273.4299999999</v>
+        <v>1350273.43</v>
       </c>
       <c r="L36">
         <v>8863</v>
@@ -4521,7 +4574,7 @@
         <v>36090.965556182942</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>59295</v>
       </c>
@@ -4595,7 +4648,7 @@
         <v>80163.138097796895</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>59299</v>
       </c>
@@ -4660,7 +4713,7 @@
         <v>2639319</v>
       </c>
       <c r="V38">
-        <v>135515.89999999999</v>
+        <v>135515.9</v>
       </c>
       <c r="W38">
         <v>0.61899999999999999</v>
@@ -4669,7 +4722,7 @@
         <v>218927.140549273</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>59301</v>
       </c>
@@ -4692,16 +4745,16 @@
         <v>303</v>
       </c>
       <c r="H39">
-        <v>2055219.1399999999</v>
+        <v>2055219.14</v>
       </c>
       <c r="I39">
-        <v>2340570.3999999999</v>
+        <v>2340570.4</v>
       </c>
       <c r="J39">
         <v>285351.25999999978</v>
       </c>
       <c r="K39">
-        <v>3172006.5600000001</v>
+        <v>3172006.56</v>
       </c>
       <c r="L39">
         <v>8135</v>
@@ -4734,7 +4787,7 @@
         <v>494481</v>
       </c>
       <c r="V39">
-        <v>99708.050000000003</v>
+        <v>99708.05</v>
       </c>
       <c r="W39">
         <v>0.49049999999999999</v>
@@ -4743,7 +4796,7 @@
         <v>203278.38939857291</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>59314</v>
       </c>
@@ -4769,7 +4822,7 @@
         <v>2266500.0499999998</v>
       </c>
       <c r="I40">
-        <v>3008670.1699999999</v>
+        <v>3008670.17</v>
       </c>
       <c r="J40">
         <v>742170.11999999965</v>
@@ -4808,7 +4861,7 @@
         <v>527151</v>
       </c>
       <c r="V40">
-        <v>94984.139999999999</v>
+        <v>94984.14</v>
       </c>
       <c r="W40">
         <v>0.73140000000000005</v>
@@ -4817,7 +4870,7 @@
         <v>129866.20180475801</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>59315</v>
       </c>
@@ -4882,7 +4935,7 @@
         <v>340055</v>
       </c>
       <c r="V41">
-        <v>150070.95999999999</v>
+        <v>150070.96</v>
       </c>
       <c r="W41">
         <v>0.53959999999999997</v>
@@ -4891,7 +4944,7 @@
         <v>278115.19644180877</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>59322</v>
       </c>
@@ -4917,7 +4970,7 @@
         <v>1558828.46</v>
       </c>
       <c r="I42">
-        <v>1587639.1100000001</v>
+        <v>1587639.11</v>
       </c>
       <c r="J42">
         <v>28810.65000000014</v>
@@ -4965,7 +5018,7 @@
         <v>186888.58290304069</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>59323</v>
       </c>
@@ -4988,7 +5041,7 @@
         <v>51</v>
       </c>
       <c r="H43">
-        <v>5293131.0800000001</v>
+        <v>5293131.08</v>
       </c>
       <c r="I43">
         <v>5389390.1299999999</v>
@@ -5030,7 +5083,7 @@
         <v>797829</v>
       </c>
       <c r="V43">
-        <v>41918.900000000001</v>
+        <v>41918.9</v>
       </c>
       <c r="W43">
         <v>0.54899999999999993</v>
@@ -5039,7 +5092,7 @@
         <v>76355.00910746814</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>59328</v>
       </c>
@@ -5113,7 +5166,7 @@
         <v>272021.48352732288</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>59336</v>
       </c>
@@ -5178,7 +5231,7 @@
         <v>2511724</v>
       </c>
       <c r="V45">
-        <v>79831.660000000003</v>
+        <v>79831.66</v>
       </c>
       <c r="W45">
         <v>0.1366</v>
@@ -5187,7 +5240,7 @@
         <v>584419.18008784775</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>59328</v>
       </c>
@@ -5261,7 +5314,7 @@
         <v>231726.46450723641</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>59332</v>
       </c>
@@ -5284,16 +5337,16 @@
         <v>332</v>
       </c>
       <c r="H47">
-        <v>1357779.4299999999</v>
+        <v>1357779.43</v>
       </c>
       <c r="I47">
-        <v>1473402.6399999999</v>
+        <v>1473402.64</v>
       </c>
       <c r="J47">
         <v>115623.2100000002</v>
       </c>
       <c r="K47">
-        <v>2293908.8500000001</v>
+        <v>2293908.85</v>
       </c>
       <c r="L47">
         <v>13201</v>
@@ -5335,7 +5388,7 @@
         <v>3242.909290016426</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>59333</v>
       </c>
@@ -5361,13 +5414,13 @@
         <v>507017.13</v>
       </c>
       <c r="I48">
-        <v>588989.41000000003</v>
+        <v>588989.41</v>
       </c>
       <c r="J48">
         <v>81972.280000000028</v>
       </c>
       <c r="K48">
-        <v>870086.98999999999</v>
+        <v>870086.99</v>
       </c>
       <c r="L48">
         <v>291</v>
@@ -5400,7 +5453,7 @@
         <v>78441</v>
       </c>
       <c r="V48">
-        <v>46673.800000000003</v>
+        <v>46673.8</v>
       </c>
       <c r="W48">
         <v>0.51800000000000002</v>
@@ -5409,7 +5462,7 @@
         <v>90103.861003861006</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>59339</v>
       </c>
@@ -5474,7 +5527,7 @@
         <v>1112189</v>
       </c>
       <c r="V49">
-        <v>73318.279999999999</v>
+        <v>73318.28</v>
       </c>
       <c r="W49">
         <v>0.62280000000000002</v>
@@ -5483,7 +5536,7 @@
         <v>117723.6351958895</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>59344</v>
       </c>
@@ -5557,7 +5610,7 @@
         <v>186094.49269222619</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>59346</v>
       </c>
@@ -5622,7 +5675,7 @@
         <v>718722</v>
       </c>
       <c r="V51">
-        <v>82185.889999999999</v>
+        <v>82185.89</v>
       </c>
       <c r="W51">
         <v>0.59889999999999999</v>
@@ -5631,7 +5684,7 @@
         <v>137228.06812489571</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>59350</v>
       </c>
@@ -5705,7 +5758,7 @@
         <v>7789751.6516516516</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>59352</v>
       </c>
@@ -5779,7 +5832,7 @@
         <v>311576.95202257758</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>59355</v>
       </c>
@@ -5802,7 +5855,7 @@
         <v>356</v>
       </c>
       <c r="H54">
-        <v>1459252.3500000001</v>
+        <v>1459252.35</v>
       </c>
       <c r="I54">
         <v>1911372.7</v>
@@ -5844,7 +5897,7 @@
         <v>362806</v>
       </c>
       <c r="V54">
-        <v>43806.389999999999</v>
+        <v>43806.39</v>
       </c>
       <c r="W54">
         <v>0.52390000000000003</v>
@@ -5853,7 +5906,7 @@
         <v>83615.938156136661</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>59360</v>
       </c>
@@ -5927,7 +5980,7 @@
         <v>107530.7833617635</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>59367</v>
       </c>
@@ -5992,7 +6045,7 @@
         <v>1890929</v>
       </c>
       <c r="V56">
-        <v>34395.690000000002</v>
+        <v>34395.69</v>
       </c>
       <c r="W56">
         <v>0.54689999999999994</v>
@@ -6001,7 +6054,7 @@
         <v>62892.100932528811</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>59368</v>
       </c>
@@ -6075,7 +6128,7 @@
         <v>1231965.5549765499</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>59386</v>
       </c>
@@ -6104,7 +6157,7 @@
         <v>17526647</v>
       </c>
       <c r="J58">
-        <v>1939148.8400000001</v>
+        <v>1939148.84</v>
       </c>
       <c r="K58">
         <v>22249813.260000002</v>
@@ -6140,7 +6193,7 @@
         <v>2082314</v>
       </c>
       <c r="V58">
-        <v>190193.32000000001</v>
+        <v>190193.32</v>
       </c>
       <c r="W58">
         <v>0.64319999999999988</v>
@@ -6149,7 +6202,7 @@
         <v>295698.56965174142</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>59387</v>
       </c>
@@ -6172,16 +6225,16 @@
         <v>388</v>
       </c>
       <c r="H59">
-        <v>1433095.3400000001</v>
+        <v>1433095.34</v>
       </c>
       <c r="I59">
-        <v>1593195.9399999999</v>
+        <v>1593195.94</v>
       </c>
       <c r="J59">
         <v>160100.59999999989</v>
       </c>
       <c r="K59">
-        <v>2363666.3300000001</v>
+        <v>2363666.33</v>
       </c>
       <c r="L59">
         <v>5816</v>
@@ -6214,7 +6267,7 @@
         <v>282116</v>
       </c>
       <c r="V59">
-        <v>100553.32000000001</v>
+        <v>100553.32</v>
       </c>
       <c r="W59">
         <v>0.56320000000000003</v>
@@ -6223,7 +6276,7 @@
         <v>178539.27556818179</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59398</v>
       </c>
@@ -6288,7 +6341,7 @@
         <v>1034932</v>
       </c>
       <c r="V60">
-        <v>32415.849999999999</v>
+        <v>32415.85</v>
       </c>
       <c r="W60">
         <v>0.48849999999999999</v>
@@ -6297,7 +6350,7 @@
         <v>66357.932446264065</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>59410</v>
       </c>
@@ -6371,7 +6424,7 @@
         <v>136802.1992818671</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>59426</v>
       </c>
@@ -6436,7 +6489,7 @@
         <v>854320</v>
       </c>
       <c r="V62">
-        <v>53613.379999999997</v>
+        <v>53613.38</v>
       </c>
       <c r="W62">
         <v>0.48380000000000001</v>
@@ -6445,7 +6498,7 @@
         <v>110817.2385283175</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>59431</v>
       </c>
@@ -6468,13 +6521,13 @@
         <v>437</v>
       </c>
       <c r="H63">
-        <v>1586678.5800000001</v>
+        <v>1586678.58</v>
       </c>
       <c r="I63">
         <v>2023576.78</v>
       </c>
       <c r="J63">
-        <v>436898.20000000001</v>
+        <v>436898.2</v>
       </c>
       <c r="K63">
         <v>5406277.6199999992</v>
@@ -6519,7 +6572,7 @@
         <v>52406.883867577497</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>59462</v>
       </c>
@@ -6584,7 +6637,7 @@
         <v>1070341</v>
       </c>
       <c r="V64">
-        <v>30117.880000000001</v>
+        <v>30117.88</v>
       </c>
       <c r="W64">
         <v>0.77879999999999994</v>
@@ -6593,7 +6646,7 @@
         <v>38672.162300975862</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>59464</v>
       </c>
@@ -6616,10 +6669,10 @@
         <v>458</v>
       </c>
       <c r="H65">
-        <v>810374.52000000002</v>
+        <v>810374.52</v>
       </c>
       <c r="I65">
-        <v>935577.33999999997</v>
+        <v>935577.34</v>
       </c>
       <c r="J65">
         <v>125202.81999999991</v>
@@ -6667,7 +6720,7 @@
         <v>16416.579144786188</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>59470</v>
       </c>
@@ -6690,10 +6743,10 @@
         <v>470</v>
       </c>
       <c r="H66">
-        <v>1565204.9099999999</v>
+        <v>1565204.91</v>
       </c>
       <c r="I66">
-        <v>1691711.1000000001</v>
+        <v>1691711.1</v>
       </c>
       <c r="J66">
         <v>126506.1899999999</v>
@@ -6732,7 +6785,7 @@
         <v>156064</v>
       </c>
       <c r="V66">
-        <v>79790.809999999998</v>
+        <v>79790.81</v>
       </c>
       <c r="W66">
         <v>0.59810000000000008</v>
@@ -6741,7 +6794,7 @@
         <v>133407.13927436879</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>59473</v>
       </c>
@@ -6764,7 +6817,7 @@
         <v>477</v>
       </c>
       <c r="H67">
-        <v>3801973.7400000002</v>
+        <v>3801973.74</v>
       </c>
       <c r="I67">
         <v>3958074</v>
@@ -6773,7 +6826,7 @@
         <v>156100.26000000021</v>
       </c>
       <c r="K67">
-        <v>3857935.0299999998</v>
+        <v>3857935.03</v>
       </c>
       <c r="L67">
         <v>21139</v>
@@ -6806,7 +6859,7 @@
         <v>455651</v>
       </c>
       <c r="V67">
-        <v>36514.459999999999</v>
+        <v>36514.46</v>
       </c>
       <c r="W67">
         <v>0.55459999999999998</v>
@@ -6815,7 +6868,7 @@
         <v>65839.27154706094</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>59484</v>
       </c>
@@ -6880,7 +6933,7 @@
         <v>962684</v>
       </c>
       <c r="V68">
-        <v>207351.70999999999</v>
+        <v>207351.71</v>
       </c>
       <c r="W68">
         <v>0.65709999999999991</v>
@@ -6889,7 +6942,7 @@
         <v>315555.79059503891</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>59495</v>
       </c>
@@ -6912,10 +6965,10 @@
         <v>487</v>
       </c>
       <c r="H69">
-        <v>940164.72999999998</v>
+        <v>940164.73</v>
       </c>
       <c r="I69">
-        <v>1127734.8100000001</v>
+        <v>1127734.81</v>
       </c>
       <c r="J69">
         <v>187570.0800000001</v>
@@ -6954,7 +7007,7 @@
         <v>89985</v>
       </c>
       <c r="V69">
-        <v>76888.139999999999</v>
+        <v>76888.14</v>
       </c>
       <c r="W69">
         <v>0.31140000000000001</v>
@@ -6963,7 +7016,7 @@
         <v>246911.1753371869</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>59503</v>
       </c>
@@ -6992,7 +7045,7 @@
         <v>21893157.760000002</v>
       </c>
       <c r="J70">
-        <v>2059264.8200000001</v>
+        <v>2059264.82</v>
       </c>
       <c r="K70">
         <v>27021885.75</v>
@@ -7037,7 +7090,7 @@
         <v>227683.2766825289</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>59507</v>
       </c>
@@ -7066,7 +7119,7 @@
         <v>18069931.199999999</v>
       </c>
       <c r="J71">
-        <v>2234205.4199999999</v>
+        <v>2234205.42</v>
       </c>
       <c r="K71">
         <v>25882677.899999999</v>
@@ -7111,7 +7164,7 @@
         <v>274860.45046764647</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>59512</v>
       </c>
@@ -7176,7 +7229,7 @@
         <v>6015537</v>
       </c>
       <c r="V72">
-        <v>300604.73999999999</v>
+        <v>300604.74</v>
       </c>
       <c r="W72">
         <v>0.60740000000000005</v>
@@ -7185,7 +7238,7 @@
         <v>494904.08297662158</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>59550</v>
       </c>
@@ -7208,16 +7261,16 @@
         <v>522</v>
       </c>
       <c r="H73">
-        <v>1744806.1799999999</v>
+        <v>1744806.18</v>
       </c>
       <c r="I73">
-        <v>2000172.9399999999</v>
+        <v>2000172.94</v>
       </c>
       <c r="J73">
-        <v>255366.76000000001</v>
+        <v>255366.76</v>
       </c>
       <c r="K73">
-        <v>2626249.3399999999</v>
+        <v>2626249.34</v>
       </c>
       <c r="L73">
         <v>6198</v>
@@ -7250,7 +7303,7 @@
         <v>482126</v>
       </c>
       <c r="V73">
-        <v>62794.059999999998</v>
+        <v>62794.06</v>
       </c>
       <c r="W73">
         <v>0.55059999999999998</v>
@@ -7259,7 +7312,7 @@
         <v>114046.603705049</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>59551</v>
       </c>
@@ -7285,7 +7338,7 @@
         <v>2695268</v>
       </c>
       <c r="I74">
-        <v>2992476.0600000001</v>
+        <v>2992476.06</v>
       </c>
       <c r="J74">
         <v>297208.06000000011</v>
@@ -7333,7 +7386,7 @@
         <v>360795.96069868997</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>59552</v>
       </c>
@@ -7407,7 +7460,7 @@
         <v>156705.08083140879</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>59553</v>
       </c>
@@ -7430,16 +7483,16 @@
         <v>550</v>
       </c>
       <c r="H76">
-        <v>2690944.7599999998</v>
+        <v>2690944.76</v>
       </c>
       <c r="I76">
-        <v>3752316.8100000001</v>
+        <v>3752316.81</v>
       </c>
       <c r="J76">
         <v>1061372.05</v>
       </c>
       <c r="K76">
-        <v>3833593.7999999998</v>
+        <v>3833593.8</v>
       </c>
       <c r="L76">
         <v>159735</v>
@@ -7472,7 +7525,7 @@
         <v>402232</v>
       </c>
       <c r="V76">
-        <v>80396.389999999999</v>
+        <v>80396.39</v>
       </c>
       <c r="W76">
         <v>0.99390000000000001</v>
@@ -7481,7 +7534,7 @@
         <v>80889.81788912366</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>59554</v>
       </c>
@@ -7504,13 +7557,13 @@
         <v>553</v>
       </c>
       <c r="H77">
-        <v>5066844.8799999999</v>
+        <v>5066844.88</v>
       </c>
       <c r="I77">
-        <v>5239118.5899999999</v>
+        <v>5239118.59</v>
       </c>
       <c r="J77">
-        <v>172273.70999999999</v>
+        <v>172273.71</v>
       </c>
       <c r="K77">
         <v>9576024.6500000004</v>
@@ -7555,7 +7608,7 @@
         <v>116788.7980932925</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>59557</v>
       </c>
@@ -7584,7 +7637,7 @@
         <v>21902392</v>
       </c>
       <c r="J78">
-        <v>1169003.8200000001</v>
+        <v>1169003.82</v>
       </c>
       <c r="K78">
         <v>30290045.489999998</v>
@@ -7623,13 +7676,13 @@
         <v>250266</v>
       </c>
       <c r="W78">
-        <v>0.42999999999999999</v>
+        <v>0.43</v>
       </c>
       <c r="X78">
         <v>582013.95348837215</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>59560</v>
       </c>
@@ -7655,7 +7708,7 @@
         <v>4300400.8499999996</v>
       </c>
       <c r="I79">
-        <v>5143975.0800000001</v>
+        <v>5143975.08</v>
       </c>
       <c r="J79">
         <v>843574.23000000045</v>
@@ -7694,7 +7747,7 @@
         <v>1184968</v>
       </c>
       <c r="V79">
-        <v>56813.129999999997</v>
+        <v>56813.13</v>
       </c>
       <c r="W79">
         <v>0.69129999999999991</v>
@@ -7703,7 +7756,7 @@
         <v>82183.031968754527</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>59563</v>
       </c>
@@ -7768,7 +7821,7 @@
         <v>3491557</v>
       </c>
       <c r="V80">
-        <v>88688.199999999997</v>
+        <v>88688.2</v>
       </c>
       <c r="W80">
         <v>0.30199999999999999</v>
@@ -7777,7 +7830,7 @@
         <v>293669.53642384108</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>59564</v>
       </c>
@@ -7800,10 +7853,10 @@
         <v>585</v>
       </c>
       <c r="H81">
-        <v>4076359.5899999999</v>
+        <v>4076359.59</v>
       </c>
       <c r="I81">
-        <v>4409456.8399999999</v>
+        <v>4409456.84</v>
       </c>
       <c r="J81">
         <v>333097.25</v>
@@ -7842,7 +7895,7 @@
         <v>67188</v>
       </c>
       <c r="V81">
-        <v>68306.309999999998</v>
+        <v>68306.31</v>
       </c>
       <c r="W81">
         <v>0.46310000000000001</v>
@@ -7851,7 +7904,7 @@
         <v>147497.97020082051</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>59586</v>
       </c>
@@ -7874,10 +7927,10 @@
         <v>598</v>
       </c>
       <c r="H82">
-        <v>2791430.1600000001</v>
+        <v>2791430.16</v>
       </c>
       <c r="I82">
-        <v>3196860.1000000001</v>
+        <v>3196860.1</v>
       </c>
       <c r="J82">
         <v>405429.93999999989</v>
@@ -7925,7 +7978,7 @@
         <v>116360.25791324741</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>59599</v>
       </c>
@@ -7999,7 +8052,7 @@
         <v>430936.36363636359</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>59600</v>
       </c>
@@ -8025,13 +8078,13 @@
         <v>1222028.26</v>
       </c>
       <c r="I84">
-        <v>1365649.6799999999</v>
+        <v>1365649.68</v>
       </c>
       <c r="J84">
         <v>143621.4199999999</v>
       </c>
       <c r="K84">
-        <v>1964631.6299999999</v>
+        <v>1964631.63</v>
       </c>
       <c r="L84">
         <v>2577</v>
@@ -8064,7 +8117,7 @@
         <v>100816</v>
       </c>
       <c r="V84">
-        <v>19006.040000000001</v>
+        <v>19006.04</v>
       </c>
       <c r="W84">
         <v>0.6604000000000001</v>
@@ -8073,7 +8126,7 @@
         <v>28779.58812840702</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>59610</v>
       </c>
@@ -8099,13 +8152,13 @@
         <v>1673858.24</v>
       </c>
       <c r="I85">
-        <v>2103020.8500000001</v>
+        <v>2103020.85</v>
       </c>
       <c r="J85">
         <v>429162.6100000001</v>
       </c>
       <c r="K85">
-        <v>3144930.9199999999</v>
+        <v>3144930.92</v>
       </c>
       <c r="L85">
         <v>7870</v>
@@ -8147,7 +8200,7 @@
         <v>57183.953557606423</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>59646</v>
       </c>
@@ -8170,7 +8223,7 @@
         <v>611</v>
       </c>
       <c r="H86">
-        <v>1903021.3500000001</v>
+        <v>1903021.35</v>
       </c>
       <c r="I86">
         <v>2278511.9700000002</v>
@@ -8179,7 +8232,7 @@
         <v>375490.62000000029</v>
       </c>
       <c r="K86">
-        <v>4233052.9500000002</v>
+        <v>4233052.95</v>
       </c>
       <c r="L86">
         <v>11436</v>
@@ -8221,7 +8274,7 @@
         <v>362364.35834020341</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>59650</v>
       </c>
@@ -8286,7 +8339,7 @@
         <v>2478207</v>
       </c>
       <c r="V87">
-        <v>476906.03999999998</v>
+        <v>476906.04</v>
       </c>
       <c r="W87">
         <v>0.87040000000000006</v>
@@ -8295,7 +8348,7 @@
         <v>547915.9466911765</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>59650</v>
       </c>
@@ -8369,7 +8422,7 @@
         <v>438498.21428571432</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>59650</v>
       </c>
@@ -8398,7 +8451,7 @@
         <v>217169.56</v>
       </c>
       <c r="J89">
-        <v>30446.310000000001</v>
+        <v>30446.31</v>
       </c>
       <c r="K89">
         <v>595151.36800000002</v>
@@ -8434,7 +8487,7 @@
         <v>114501</v>
       </c>
       <c r="V89">
-        <v>44952.620000000003</v>
+        <v>44952.62</v>
       </c>
       <c r="W89">
         <v>0.22620000000000001</v>
@@ -8443,7 +8496,7 @@
         <v>198729.5313881521</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>59656</v>
       </c>
@@ -8517,7 +8570,7 @@
         <v>344246.97706740792</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>59660</v>
       </c>
@@ -8591,7 +8644,7 @@
         <v>142505.94604514589</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>59657</v>
       </c>
@@ -8656,7 +8709,7 @@
         <v>6149788</v>
       </c>
       <c r="V92">
-        <v>338605.03999999998</v>
+        <v>338605.04</v>
       </c>
       <c r="W92">
         <v>1.1304000000000001</v>
@@ -8665,7 +8718,7 @@
         <v>299544.44444444438</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>59602</v>
       </c>
@@ -8739,7 +8792,7 @@
         <v>311686.90176322422</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>59643</v>
       </c>
@@ -8804,7 +8857,7 @@
         <v>953326</v>
       </c>
       <c r="V94">
-        <v>92075.699999999997</v>
+        <v>92075.7</v>
       </c>
       <c r="W94">
         <v>0.57700000000000007</v>
@@ -8813,7 +8866,7 @@
         <v>159576.603119584</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>59646</v>
       </c>
@@ -8839,7 +8892,7 @@
         <v>318013.78000000003</v>
       </c>
       <c r="I95">
-        <v>427765.79999999999</v>
+        <v>427765.8</v>
       </c>
       <c r="J95">
         <v>109752.02</v>
@@ -8878,7 +8931,7 @@
         <v>97759</v>
       </c>
       <c r="V95">
-        <v>44870.790000000001</v>
+        <v>44870.79</v>
       </c>
       <c r="W95">
         <v>0.71790000000000009</v>
@@ -8887,7 +8940,7 @@
         <v>62502.841621395732</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>59658</v>
       </c>
@@ -8913,13 +8966,13 @@
         <v>2447853.77</v>
       </c>
       <c r="I96">
-        <v>3052563.8799999999</v>
+        <v>3052563.88</v>
       </c>
       <c r="J96">
         <v>604710.10999999987</v>
       </c>
       <c r="K96">
-        <v>4087240.4399999999</v>
+        <v>4087240.44</v>
       </c>
       <c r="L96">
         <v>3324</v>

</xml_diff>